<commit_message>
Dimplex and La Redoute links across 5 guides; Awin tracker: 2 approvals, 5 rejections
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UM6BC1UkD1TGZjj46L45Yj
</commit_message>
<xml_diff>
--- a/ops/awin-applications.xlsx
+++ b/ops/awin-applications.xlsx
@@ -657,11 +657,19 @@
       </c>
       <c r="I7" s="16" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="J7" s="16" t="n"/>
-      <c r="K7" s="14" t="n"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="K7" s="14" t="inlineStr">
+        <is>
+          <t>Live: stay-warm heaters (2), Black Friday radiator.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="10">
       <c r="A8" s="14" t="n">
@@ -884,13 +892,17 @@
       </c>
       <c r="I12" s="16" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="J12" s="16" t="n"/>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="J12" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
       <c r="K12" s="14" t="inlineStr">
         <is>
-          <t>No buy-now-pay-later publishers (not us)</t>
+          <t>Reason: content focus/audience not aligned with Currys range or customers</t>
         </is>
       </c>
     </row>
@@ -931,11 +943,19 @@
       </c>
       <c r="I13" s="16" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="J13" s="16" t="n"/>
-      <c r="K13" s="14" t="n"/>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Reason: site does not complement advertiser brand</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="10">
       <c r="A14" s="14" t="n">
@@ -1107,11 +1127,19 @@
       </c>
       <c r="I17" s="16" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="J17" s="16" t="n"/>
-      <c r="K17" s="14" t="n"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="K17" s="14" t="inlineStr">
+        <is>
+          <t>Live: living room (5), stay-warm curtains/rug (3), gifts curtains, Black Friday (2). AM: laredoute@accelerationpartners.com</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="10">
       <c r="A18" s="14" t="n">
@@ -1287,11 +1315,19 @@
       </c>
       <c r="I21" s="16" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="J21" s="16" t="n"/>
-      <c r="K21" s="14" t="n"/>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="J21" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="K21" s="14" t="inlineStr">
+        <is>
+          <t>Reason: site does not complement advertiser brand</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="10">
       <c r="A22" s="14" t="n">
@@ -1330,11 +1366,19 @@
       </c>
       <c r="I22" s="16" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="J22" s="16" t="n"/>
-      <c r="K22" s="14" t="n"/>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="J22" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="K22" s="14" t="inlineStr">
+        <is>
+          <t>Reason: URL is irrelevant to advertiser brand</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="23.85" customHeight="1" s="10">
       <c r="A23" s="14" t="n">
@@ -1373,13 +1417,17 @@
       </c>
       <c r="I23" s="16" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="J23" s="16" t="n"/>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="J23" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
       <c r="K23" s="14" t="inlineStr">
         <is>
-          <t>Rate depends on new/existing and cash/credit customer</t>
+          <t>Reason: site does not complement advertiser brand</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Board meeting 18 Oct: plan register (manager playbook), Meaco links, Awin tracker update
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014oiBn3GRWoXm1MgCErKnBr
</commit_message>
<xml_diff>
--- a/ops/awin-applications.xlsx
+++ b/ops/awin-applications.xlsx
@@ -614,11 +614,19 @@
       </c>
       <c r="I6" s="16" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="J6" s="16" t="n"/>
-      <c r="K6" s="14" t="n"/>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="J6" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>Live: dehumidifiers guide (Arete One, DD8L Zambezi, desiccant range) – added 18 Oct.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="10">
       <c r="A7" s="14" t="n">
@@ -1041,11 +1049,19 @@
       </c>
       <c r="I15" s="16" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="J15" s="16" t="n"/>
-      <c r="K15" s="14" t="n"/>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="K15" s="14" t="inlineStr">
+        <is>
+          <t>Rejected 15 Oct (reason in Awin email: asked to apply via another route – see email).</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="10">
       <c r="A16" s="14" t="n">
@@ -1137,7 +1153,7 @@
       </c>
       <c r="K17" s="14" t="inlineStr">
         <is>
-          <t>Live: living room (5), stay-warm curtains/rug (3), gifts curtains, Black Friday (2). AM: laredoute@accelerationpartners.com</t>
+          <t>Live: living room (5), stay-warm curtains/rug (3), gifts curtains, Black Friday (2). AM: laredoute@accelerationpartners.com Commission rates changed 17 Oct (Awin email) – check new rate in Awin.</t>
         </is>
       </c>
     </row>
@@ -1474,6 +1490,7 @@
         </is>
       </c>
     </row>
+    <row r="25"/>
     <row r="26" ht="15" customHeight="1" s="10">
       <c r="H26" s="17" t="inlineStr">
         <is>
@@ -1518,6 +1535,7 @@
         <v/>
       </c>
     </row>
+    <row r="30"/>
     <row r="31" ht="15" customHeight="1" s="10">
       <c r="A31" s="12" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Awin checked after sign-in: 5 clicks Oct, La Redoute 2-4%; register #23 done
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HAESKjBjXMEBgnHQXhDcwE
</commit_message>
<xml_diff>
--- a/ops/awin-applications.xlsx
+++ b/ops/awin-applications.xlsx
@@ -1120,7 +1120,7 @@
       </c>
       <c r="D17" s="15" t="inlineStr">
         <is>
-          <t>Not shown</t>
+          <t>2%–4% (Awin commission timeline, 19 Oct)</t>
         </is>
       </c>
       <c r="E17" s="15" t="n">
@@ -1153,7 +1153,7 @@
       </c>
       <c r="K17" s="14" t="inlineStr">
         <is>
-          <t>Live: living room (5), stay-warm curtains/rug (3), gifts curtains, Black Friday (2). AM: laredoute@accelerationpartners.com Commission rates changed 17 Oct (Awin email) – check new rate in Awin.</t>
+          <t>Live: living room (5), stay-warm curtains/rug (3), gifts curtains, Black Friday (2). AM: laredoute@accelerationpartners.com. Rates changed 17 Oct – now 2%–4% (checked 19 Oct). Awin shows payment "Exposure Level 2" (advertiser over credit limit), avg payment 85 days – commission may be slow to pay.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CEO report 30 Oct (on request): AO rejected, register #51 GoatCounter access, #52 Homebase BF links, #2 hold pending #39
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SEh8HUSDJr4WqHRw4HqnJ9
</commit_message>
<xml_diff>
--- a/ops/awin-applications.xlsx
+++ b/ops/awin-applications.xlsx
@@ -857,11 +857,19 @@
       </c>
       <c r="I11" s="16" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="J11" s="16" t="n"/>
-      <c r="K11" s="14" t="n"/>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="K11" s="14" t="inlineStr">
+        <is>
+          <t>Reason (Awin email 29 Oct): site does not complement advertiser brand</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="10">
       <c r="A12" s="14" t="n">
@@ -1490,7 +1498,6 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
     <row r="26" ht="15" customHeight="1" s="10">
       <c r="H26" s="17" t="inlineStr">
         <is>
@@ -1535,7 +1542,6 @@
         <v/>
       </c>
     </row>
-    <row r="30"/>
     <row r="31" ht="15" customHeight="1" s="10">
       <c r="A31" s="12" t="inlineStr">
         <is>

</xml_diff>